<commit_message>
Feat: Add gui interface and BATCH_DESC
</commit_message>
<xml_diff>
--- a/test/if-batch-message-flow/commands_sample_if_batch.xlsx
+++ b/test/if-batch-message-flow/commands_sample_if_batch.xlsx
@@ -559,6 +559,23 @@
           <t>BATCH_START(AccountAudit)</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Input Schema:
+{
+  "target_user": {
+    "type": "string",
+    "required": true,
+    "description": "Target account username for the audit batch"
+  },
+  "from_status": {
+    "type": "integer",
+    "required": false,
+    "description": "Status code propagated from the outer flow"
+  }
+}</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -642,7 +659,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -655,7 +671,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
@@ -673,7 +688,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>

</xml_diff>